<commit_message>
Copy audit, script and data text: no talk of how figures were read or checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012JjD5mhtvLxzAXoZHMZYE5
</commit_message>
<xml_diff>
--- a/downloads/other-states.xlsx
+++ b/downloads/other-states.xlsx
@@ -647,7 +647,7 @@
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>How many names were left off in any ward or sector. The Chief Electoral Officer's site could not be reached and no table below the union territory was found. A ward table that newspapers reported from a chart shared by the member of parliament. It compares the roll of the 2024 Lok Sabha election with a later roll, two years apart, and gives a percentage for most wards and a count for only six, for 17 of the 35 wards. The chart's own date is reported as 2 August 2026 and the chart itself was not found, so it is left out. The draft by sex and the names left off by sex. They were reported in one news agency story that could not be read, so they are left out. How many of the 15,117 names added after the draft were people left off it.</t>
+          <t>How many names were left off in any ward or sector. No table below the union territory was found. A ward table that newspapers reported from a chart shared by the member of parliament. It compares the roll of the 2024 Lok Sabha election with a later roll, two years apart, and gives a percentage for most wards and a count for only six, for 17 of the 35 wards. The chart's own date is reported as 2 August 2026 and the chart itself was not found, so it is left out. The draft by sex and the names left off by sex. They were reported in one news agency story whose text is not available, so they are left out. How many of the 15,117 names added after the draft were people left off it.</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>There are no figures yet. The roll before the revision, the names left off and their reasons will be known only when the draft is published. The Chief Electoral Officer's site could not be reached, so nothing was read from it.</t>
+          <t>There are no figures yet. The roll before the revision, the names left off and their reasons will be known only when the draft is published.</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Meghalaya final roll of 26 October, template wording, India report, first reading (second reading in progress)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012JjD5mhtvLxzAXoZHMZYE5
</commit_message>
<xml_diff>
--- a/downloads/other-states.xlsx
+++ b/downloads/other-states.xlsx
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Women's share of the names left off in any district or constituency. The roll by sex was published for the state only. Where the notices and hearings fell. They were published as state totals only. The final roll, which was not out when these figures were read.</t>
+          <t>Women's share of the names left off in any district or constituency. The roll by sex was published for the state only. Where the notices and hearings fell, and where names were added or deleted after the draft. They were published as state totals only. The final roll by district or constituency. The note of 26 October 2026 gives it for the state only, so the district and constituency figures stop at the draft. How many of the 21,694 electors added on Form 6 or 6A had been left off the draft and how many were new voters.</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
@@ -8232,7 +8232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S89"/>
+  <dimension ref="A1:S96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8816,15 +8816,15 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>notices</t>
+          <t>added_after</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>651735</v>
+        <v>23970</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/87 of 1 October 2026</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -8836,48 +8836,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>West Jaintia Hills</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>220478</v>
-      </c>
-      <c r="F18" t="n">
-        <v>209908</v>
-      </c>
-      <c r="G18" t="n">
-        <v>10570</v>
-      </c>
-      <c r="N18" t="n">
-        <v>7097</v>
-      </c>
-      <c r="O18" t="n">
-        <v>3151</v>
-      </c>
-      <c r="P18" t="n">
-        <v>322</v>
+          <t>removed_after</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>9250</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S18" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8886,48 +8866,28 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ri-Bhoi</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>205735</v>
-      </c>
-      <c r="F19" t="n">
-        <v>190066</v>
-      </c>
-      <c r="G19" t="n">
-        <v>15669</v>
-      </c>
-      <c r="N19" t="n">
-        <v>6096</v>
-      </c>
-      <c r="O19" t="n">
-        <v>9040</v>
-      </c>
-      <c r="P19" t="n">
-        <v>533</v>
+          <t>net_after</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>14720</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S19" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8936,48 +8896,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>East Khasi Hills</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>632146</v>
-      </c>
-      <c r="F20" t="n">
-        <v>562160</v>
-      </c>
-      <c r="G20" t="n">
-        <v>69986</v>
-      </c>
-      <c r="N20" t="n">
-        <v>27319</v>
-      </c>
-      <c r="O20" t="n">
-        <v>40940</v>
-      </c>
-      <c r="P20" t="n">
-        <v>1727</v>
+          <t>final</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>2183963</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S20" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -8986,48 +8926,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>West Khasi Hills</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>137727</v>
-      </c>
-      <c r="F21" t="n">
-        <v>129820</v>
-      </c>
-      <c r="G21" t="n">
-        <v>7907</v>
-      </c>
-      <c r="N21" t="n">
-        <v>4455</v>
-      </c>
-      <c r="O21" t="n">
-        <v>3013</v>
-      </c>
-      <c r="P21" t="n">
-        <v>439</v>
+          <t>men_final</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1059743</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S21" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9036,48 +8956,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>East Garo Hills</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>114767</v>
-      </c>
-      <c r="F22" t="n">
-        <v>105512</v>
-      </c>
-      <c r="G22" t="n">
-        <v>9255</v>
-      </c>
-      <c r="N22" t="n">
-        <v>2905</v>
-      </c>
-      <c r="O22" t="n">
-        <v>5761</v>
-      </c>
-      <c r="P22" t="n">
-        <v>589</v>
+          <t>women_final</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1124216</v>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9086,48 +8986,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>West Garo Hills</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>396914</v>
-      </c>
-      <c r="F23" t="n">
-        <v>367382</v>
-      </c>
-      <c r="G23" t="n">
-        <v>29532</v>
-      </c>
-      <c r="N23" t="n">
-        <v>15613</v>
-      </c>
-      <c r="O23" t="n">
-        <v>12874</v>
-      </c>
-      <c r="P23" t="n">
-        <v>1045</v>
+          <t>third_final</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S23" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9136,48 +9016,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>districts</t>
+          <t>state</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>district</t>
+          <t>state</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>South Garo Hills</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>110488</v>
-      </c>
-      <c r="F24" t="n">
-        <v>102649</v>
-      </c>
-      <c r="G24" t="n">
-        <v>7839</v>
-      </c>
-      <c r="N24" t="n">
-        <v>3583</v>
-      </c>
-      <c r="O24" t="n">
-        <v>3782</v>
-      </c>
-      <c r="P24" t="n">
-        <v>474</v>
+          <t>notices</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>651735</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/102 of 26 October 2026 on the final roll</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S24" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -9196,26 +9056,26 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>East Jaintia Hills</t>
+          <t>West Jaintia Hills</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>104417</v>
+        <v>220478</v>
       </c>
       <c r="F25" t="n">
-        <v>96791</v>
+        <v>209908</v>
       </c>
       <c r="G25" t="n">
-        <v>7626</v>
+        <v>10570</v>
       </c>
       <c r="N25" t="n">
-        <v>3598</v>
+        <v>7097</v>
       </c>
       <c r="O25" t="n">
-        <v>3448</v>
+        <v>3151</v>
       </c>
       <c r="P25" t="n">
-        <v>580</v>
+        <v>322</v>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
@@ -9246,26 +9106,26 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>South West Khasi Hills</t>
+          <t>Ri-Bhoi</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>80592</v>
+        <v>205735</v>
       </c>
       <c r="F26" t="n">
-        <v>77124</v>
+        <v>190066</v>
       </c>
       <c r="G26" t="n">
-        <v>3468</v>
+        <v>15669</v>
       </c>
       <c r="N26" t="n">
-        <v>2305</v>
+        <v>6096</v>
       </c>
       <c r="O26" t="n">
-        <v>1017</v>
+        <v>9040</v>
       </c>
       <c r="P26" t="n">
-        <v>146</v>
+        <v>533</v>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
@@ -9296,26 +9156,26 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>North Garo Hills</t>
+          <t>East Khasi Hills</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>143748</v>
+        <v>632146</v>
       </c>
       <c r="F27" t="n">
-        <v>132013</v>
+        <v>562160</v>
       </c>
       <c r="G27" t="n">
-        <v>11735</v>
+        <v>69986</v>
       </c>
       <c r="N27" t="n">
-        <v>4578</v>
+        <v>27319</v>
       </c>
       <c r="O27" t="n">
-        <v>6769</v>
+        <v>40940</v>
       </c>
       <c r="P27" t="n">
-        <v>388</v>
+        <v>1727</v>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
@@ -9346,26 +9206,26 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>South West Garo Hills</t>
+          <t>West Khasi Hills</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>108883</v>
+        <v>137727</v>
       </c>
       <c r="F28" t="n">
-        <v>104671</v>
+        <v>129820</v>
       </c>
       <c r="G28" t="n">
-        <v>4212</v>
+        <v>7907</v>
       </c>
       <c r="N28" t="n">
-        <v>2478</v>
+        <v>4455</v>
       </c>
       <c r="O28" t="n">
-        <v>1428</v>
+        <v>3013</v>
       </c>
       <c r="P28" t="n">
-        <v>306</v>
+        <v>439</v>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
@@ -9396,26 +9256,26 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Eastern West Khasi Hills</t>
+          <t>East Garo Hills</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>93750</v>
+        <v>114767</v>
       </c>
       <c r="F29" t="n">
-        <v>91147</v>
+        <v>105512</v>
       </c>
       <c r="G29" t="n">
-        <v>2603</v>
+        <v>9255</v>
       </c>
       <c r="N29" t="n">
-        <v>1463</v>
+        <v>2905</v>
       </c>
       <c r="O29" t="n">
-        <v>988</v>
+        <v>5761</v>
       </c>
       <c r="P29" t="n">
-        <v>152</v>
+        <v>589</v>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
@@ -9436,36 +9296,36 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1 Nartiang</t>
+          <t>West Garo Hills</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>48718</v>
+        <v>396914</v>
       </c>
       <c r="F30" t="n">
-        <v>46104</v>
+        <v>367382</v>
       </c>
       <c r="G30" t="n">
-        <v>2614</v>
+        <v>29532</v>
       </c>
       <c r="N30" t="n">
-        <v>1807</v>
+        <v>15613</v>
       </c>
       <c r="O30" t="n">
-        <v>722</v>
+        <v>12874</v>
       </c>
       <c r="P30" t="n">
-        <v>85</v>
+        <v>1045</v>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
@@ -9486,36 +9346,36 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2 Jowai</t>
+          <t>South Garo Hills</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>43838</v>
+        <v>110488</v>
       </c>
       <c r="F31" t="n">
-        <v>41521</v>
+        <v>102649</v>
       </c>
       <c r="G31" t="n">
-        <v>2317</v>
+        <v>7839</v>
       </c>
       <c r="N31" t="n">
-        <v>1437</v>
+        <v>3583</v>
       </c>
       <c r="O31" t="n">
-        <v>795</v>
+        <v>3782</v>
       </c>
       <c r="P31" t="n">
-        <v>85</v>
+        <v>474</v>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
@@ -9536,36 +9396,36 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3 Raliang</t>
+          <t>East Jaintia Hills</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>42961</v>
+        <v>104417</v>
       </c>
       <c r="F32" t="n">
-        <v>40927</v>
+        <v>96791</v>
       </c>
       <c r="G32" t="n">
-        <v>2034</v>
+        <v>7626</v>
       </c>
       <c r="N32" t="n">
-        <v>1635</v>
+        <v>3598</v>
       </c>
       <c r="O32" t="n">
-        <v>361</v>
+        <v>3448</v>
       </c>
       <c r="P32" t="n">
-        <v>38</v>
+        <v>580</v>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
@@ -9586,36 +9446,36 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4 Mowkaiaw</t>
+          <t>South West Khasi Hills</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>42837</v>
+        <v>80592</v>
       </c>
       <c r="F33" t="n">
-        <v>40706</v>
+        <v>77124</v>
       </c>
       <c r="G33" t="n">
-        <v>2131</v>
+        <v>3468</v>
       </c>
       <c r="N33" t="n">
-        <v>1260</v>
+        <v>2305</v>
       </c>
       <c r="O33" t="n">
-        <v>774</v>
+        <v>1017</v>
       </c>
       <c r="P33" t="n">
-        <v>97</v>
+        <v>146</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -9636,36 +9496,36 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>5 Sutnga Saipung</t>
+          <t>North Garo Hills</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>51956</v>
+        <v>143748</v>
       </c>
       <c r="F34" t="n">
-        <v>48631</v>
+        <v>132013</v>
       </c>
       <c r="G34" t="n">
-        <v>3325</v>
+        <v>11735</v>
       </c>
       <c r="N34" t="n">
-        <v>1614</v>
+        <v>4578</v>
       </c>
       <c r="O34" t="n">
-        <v>1390</v>
+        <v>6769</v>
       </c>
       <c r="P34" t="n">
-        <v>321</v>
+        <v>388</v>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
@@ -9686,36 +9546,36 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>6 Khliehriat</t>
+          <t>South West Garo Hills</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>52461</v>
+        <v>108883</v>
       </c>
       <c r="F35" t="n">
-        <v>48160</v>
+        <v>104671</v>
       </c>
       <c r="G35" t="n">
-        <v>4301</v>
+        <v>4212</v>
       </c>
       <c r="N35" t="n">
-        <v>1984</v>
+        <v>2478</v>
       </c>
       <c r="O35" t="n">
-        <v>2058</v>
+        <v>1428</v>
       </c>
       <c r="P35" t="n">
-        <v>259</v>
+        <v>306</v>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
@@ -9736,36 +9596,36 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>constituencies</t>
+          <t>districts</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ac</t>
+          <t>district</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>7 Amlarem</t>
+          <t>Eastern West Khasi Hills</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>42124</v>
+        <v>93750</v>
       </c>
       <c r="F36" t="n">
-        <v>40650</v>
+        <v>91147</v>
       </c>
       <c r="G36" t="n">
-        <v>1474</v>
+        <v>2603</v>
       </c>
       <c r="N36" t="n">
-        <v>958</v>
+        <v>1463</v>
       </c>
       <c r="O36" t="n">
-        <v>499</v>
+        <v>988</v>
       </c>
       <c r="P36" t="n">
-        <v>17</v>
+        <v>152</v>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
@@ -9796,26 +9656,26 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>8 Mawhati</t>
+          <t>1 Nartiang</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>42861</v>
+        <v>48718</v>
       </c>
       <c r="F37" t="n">
-        <v>40960</v>
+        <v>46104</v>
       </c>
       <c r="G37" t="n">
-        <v>1901</v>
+        <v>2614</v>
       </c>
       <c r="N37" t="n">
-        <v>1027</v>
+        <v>1807</v>
       </c>
       <c r="O37" t="n">
-        <v>793</v>
+        <v>722</v>
       </c>
       <c r="P37" t="n">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
@@ -9846,26 +9706,26 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>9 Nongpoh</t>
+          <t>2 Jowai</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>40943</v>
+        <v>43838</v>
       </c>
       <c r="F38" t="n">
-        <v>38528</v>
+        <v>41521</v>
       </c>
       <c r="G38" t="n">
-        <v>2415</v>
+        <v>2317</v>
       </c>
       <c r="N38" t="n">
-        <v>1104</v>
+        <v>1437</v>
       </c>
       <c r="O38" t="n">
-        <v>1207</v>
+        <v>795</v>
       </c>
       <c r="P38" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -9896,26 +9756,26 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>10 Jirang</t>
+          <t>3 Raliang</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>44173</v>
+        <v>42961</v>
       </c>
       <c r="F39" t="n">
-        <v>38734</v>
+        <v>40927</v>
       </c>
       <c r="G39" t="n">
-        <v>5439</v>
+        <v>2034</v>
       </c>
       <c r="N39" t="n">
-        <v>1306</v>
+        <v>1635</v>
       </c>
       <c r="O39" t="n">
-        <v>4038</v>
+        <v>361</v>
       </c>
       <c r="P39" t="n">
-        <v>95</v>
+        <v>38</v>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
@@ -9946,26 +9806,26 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11 Umsning</t>
+          <t>4 Mowkaiaw</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>42386</v>
+        <v>42837</v>
       </c>
       <c r="F40" t="n">
-        <v>39105</v>
+        <v>40706</v>
       </c>
       <c r="G40" t="n">
-        <v>3281</v>
+        <v>2131</v>
       </c>
       <c r="N40" t="n">
-        <v>1459</v>
+        <v>1260</v>
       </c>
       <c r="O40" t="n">
-        <v>1667</v>
+        <v>774</v>
       </c>
       <c r="P40" t="n">
-        <v>155</v>
+        <v>97</v>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
@@ -9996,26 +9856,26 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>12 Umroi</t>
+          <t>5 Sutnga Saipung</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>35372</v>
+        <v>51956</v>
       </c>
       <c r="F41" t="n">
-        <v>32739</v>
+        <v>48631</v>
       </c>
       <c r="G41" t="n">
-        <v>2633</v>
+        <v>3325</v>
       </c>
       <c r="N41" t="n">
-        <v>1200</v>
+        <v>1614</v>
       </c>
       <c r="O41" t="n">
-        <v>1335</v>
+        <v>1390</v>
       </c>
       <c r="P41" t="n">
-        <v>98</v>
+        <v>321</v>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
@@ -10046,26 +9906,26 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>13 Mawryngkneng</t>
+          <t>6 Khliehriat</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>43706</v>
+        <v>52461</v>
       </c>
       <c r="F42" t="n">
-        <v>40504</v>
+        <v>48160</v>
       </c>
       <c r="G42" t="n">
-        <v>3202</v>
+        <v>4301</v>
       </c>
       <c r="N42" t="n">
-        <v>1976</v>
+        <v>1984</v>
       </c>
       <c r="O42" t="n">
-        <v>1073</v>
+        <v>2058</v>
       </c>
       <c r="P42" t="n">
-        <v>153</v>
+        <v>259</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -10096,26 +9956,26 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14 Pynthorumkhrah</t>
+          <t>7 Amlarem</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>36571</v>
+        <v>42124</v>
       </c>
       <c r="F43" t="n">
-        <v>29784</v>
+        <v>40650</v>
       </c>
       <c r="G43" t="n">
-        <v>6787</v>
+        <v>1474</v>
       </c>
       <c r="N43" t="n">
-        <v>1903</v>
+        <v>958</v>
       </c>
       <c r="O43" t="n">
-        <v>4758</v>
+        <v>499</v>
       </c>
       <c r="P43" t="n">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
@@ -10146,26 +10006,26 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>15 Mawlai</t>
+          <t>8 Mawhati</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>52893</v>
+        <v>42861</v>
       </c>
       <c r="F44" t="n">
-        <v>47323</v>
+        <v>40960</v>
       </c>
       <c r="G44" t="n">
-        <v>5570</v>
+        <v>1901</v>
       </c>
       <c r="N44" t="n">
-        <v>1775</v>
+        <v>1027</v>
       </c>
       <c r="O44" t="n">
-        <v>3672</v>
+        <v>793</v>
       </c>
       <c r="P44" t="n">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
@@ -10196,26 +10056,26 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16 East Shillong</t>
+          <t>9 Nongpoh</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>25300</v>
+        <v>40943</v>
       </c>
       <c r="F45" t="n">
-        <v>19692</v>
+        <v>38528</v>
       </c>
       <c r="G45" t="n">
-        <v>5608</v>
+        <v>2415</v>
       </c>
       <c r="N45" t="n">
-        <v>1419</v>
+        <v>1104</v>
       </c>
       <c r="O45" t="n">
-        <v>4134</v>
+        <v>1207</v>
       </c>
       <c r="P45" t="n">
-        <v>55</v>
+        <v>104</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -10246,26 +10106,26 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17 North Shillong</t>
+          <t>10 Jirang</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>28072</v>
+        <v>44173</v>
       </c>
       <c r="F46" t="n">
-        <v>21509</v>
+        <v>38734</v>
       </c>
       <c r="G46" t="n">
-        <v>6563</v>
+        <v>5439</v>
       </c>
       <c r="N46" t="n">
-        <v>2011</v>
+        <v>1306</v>
       </c>
       <c r="O46" t="n">
-        <v>4423</v>
+        <v>4038</v>
       </c>
       <c r="P46" t="n">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
@@ -10296,26 +10156,26 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>18 West Shillong</t>
+          <t>11 Umsning</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>27331</v>
+        <v>42386</v>
       </c>
       <c r="F47" t="n">
-        <v>21182</v>
+        <v>39105</v>
       </c>
       <c r="G47" t="n">
-        <v>6149</v>
+        <v>3281</v>
       </c>
       <c r="N47" t="n">
-        <v>1820</v>
+        <v>1459</v>
       </c>
       <c r="O47" t="n">
-        <v>4269</v>
+        <v>1667</v>
       </c>
       <c r="P47" t="n">
-        <v>60</v>
+        <v>155</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -10346,26 +10206,26 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>19 South Shillong</t>
+          <t>12 Umroi</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>34077</v>
+        <v>35372</v>
       </c>
       <c r="F48" t="n">
-        <v>26322</v>
+        <v>32739</v>
       </c>
       <c r="G48" t="n">
-        <v>7755</v>
+        <v>2633</v>
       </c>
       <c r="N48" t="n">
-        <v>1809</v>
+        <v>1200</v>
       </c>
       <c r="O48" t="n">
-        <v>5901</v>
+        <v>1335</v>
       </c>
       <c r="P48" t="n">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -10396,26 +10256,26 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>20 Mylliem</t>
+          <t>13 Mawryngkneng</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>38922</v>
+        <v>43706</v>
       </c>
       <c r="F49" t="n">
-        <v>36289</v>
+        <v>40504</v>
       </c>
       <c r="G49" t="n">
-        <v>2633</v>
+        <v>3202</v>
       </c>
       <c r="N49" t="n">
-        <v>1260</v>
+        <v>1976</v>
       </c>
       <c r="O49" t="n">
-        <v>1282</v>
+        <v>1073</v>
       </c>
       <c r="P49" t="n">
-        <v>91</v>
+        <v>153</v>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
@@ -10446,26 +10306,26 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>21 Nongthymmai</t>
+          <t>14 Pynthorumkhrah</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>36850</v>
+        <v>36571</v>
       </c>
       <c r="F50" t="n">
-        <v>29437</v>
+        <v>29784</v>
       </c>
       <c r="G50" t="n">
-        <v>7413</v>
+        <v>6787</v>
       </c>
       <c r="N50" t="n">
-        <v>2068</v>
+        <v>1903</v>
       </c>
       <c r="O50" t="n">
-        <v>5213</v>
+        <v>4758</v>
       </c>
       <c r="P50" t="n">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
@@ -10496,26 +10356,26 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>22 Nongkrem</t>
+          <t>15 Mawlai</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>40276</v>
+        <v>52893</v>
       </c>
       <c r="F51" t="n">
-        <v>37246</v>
+        <v>47323</v>
       </c>
       <c r="G51" t="n">
-        <v>3030</v>
+        <v>5570</v>
       </c>
       <c r="N51" t="n">
-        <v>1341</v>
+        <v>1775</v>
       </c>
       <c r="O51" t="n">
-        <v>1622</v>
+        <v>3672</v>
       </c>
       <c r="P51" t="n">
-        <v>67</v>
+        <v>123</v>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
@@ -10546,26 +10406,26 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>23 Sohiong</t>
+          <t>16 East Shillong</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>37496</v>
+        <v>25300</v>
       </c>
       <c r="F52" t="n">
-        <v>35223</v>
+        <v>19692</v>
       </c>
       <c r="G52" t="n">
-        <v>2273</v>
+        <v>5608</v>
       </c>
       <c r="N52" t="n">
-        <v>1212</v>
+        <v>1419</v>
       </c>
       <c r="O52" t="n">
-        <v>968</v>
+        <v>4134</v>
       </c>
       <c r="P52" t="n">
-        <v>93</v>
+        <v>55</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
@@ -10596,26 +10456,26 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>24 Mawphlang</t>
+          <t>17 North Shillong</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>38518</v>
+        <v>28072</v>
       </c>
       <c r="F53" t="n">
-        <v>36168</v>
+        <v>21509</v>
       </c>
       <c r="G53" t="n">
-        <v>2350</v>
+        <v>6563</v>
       </c>
       <c r="N53" t="n">
-        <v>1507</v>
+        <v>2011</v>
       </c>
       <c r="O53" t="n">
-        <v>675</v>
+        <v>4423</v>
       </c>
       <c r="P53" t="n">
-        <v>168</v>
+        <v>129</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
@@ -10646,26 +10506,26 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>25 Mawsynram</t>
+          <t>18 West Shillong</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>39984</v>
+        <v>27331</v>
       </c>
       <c r="F54" t="n">
-        <v>37626</v>
+        <v>21182</v>
       </c>
       <c r="G54" t="n">
-        <v>2358</v>
+        <v>6149</v>
       </c>
       <c r="N54" t="n">
-        <v>1483</v>
+        <v>1820</v>
       </c>
       <c r="O54" t="n">
-        <v>739</v>
+        <v>4269</v>
       </c>
       <c r="P54" t="n">
-        <v>136</v>
+        <v>60</v>
       </c>
       <c r="Q54" t="inlineStr">
         <is>
@@ -10696,26 +10556,26 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>26 Shella</t>
+          <t>19 South Shillong</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>37925</v>
+        <v>34077</v>
       </c>
       <c r="F55" t="n">
-        <v>35207</v>
+        <v>26322</v>
       </c>
       <c r="G55" t="n">
-        <v>2718</v>
+        <v>7755</v>
       </c>
       <c r="N55" t="n">
-        <v>1558</v>
+        <v>1809</v>
       </c>
       <c r="O55" t="n">
-        <v>1072</v>
+        <v>5901</v>
       </c>
       <c r="P55" t="n">
-        <v>88</v>
+        <v>45</v>
       </c>
       <c r="Q55" t="inlineStr">
         <is>
@@ -10746,26 +10606,26 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>27 Pynursla</t>
+          <t>20 Mylliem</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>41748</v>
+        <v>38922</v>
       </c>
       <c r="F56" t="n">
-        <v>39314</v>
+        <v>36289</v>
       </c>
       <c r="G56" t="n">
-        <v>2434</v>
+        <v>2633</v>
       </c>
       <c r="N56" t="n">
-        <v>1941</v>
+        <v>1260</v>
       </c>
       <c r="O56" t="n">
-        <v>390</v>
+        <v>1282</v>
       </c>
       <c r="P56" t="n">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="Q56" t="inlineStr">
         <is>
@@ -10796,26 +10656,26 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>28 Sohra</t>
+          <t>21 Nongthymmai</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>32220</v>
+        <v>36850</v>
       </c>
       <c r="F57" t="n">
-        <v>30532</v>
+        <v>29437</v>
       </c>
       <c r="G57" t="n">
-        <v>1688</v>
+        <v>7413</v>
       </c>
       <c r="N57" t="n">
-        <v>1329</v>
+        <v>2068</v>
       </c>
       <c r="O57" t="n">
-        <v>313</v>
+        <v>5213</v>
       </c>
       <c r="P57" t="n">
-        <v>46</v>
+        <v>132</v>
       </c>
       <c r="Q57" t="inlineStr">
         <is>
@@ -10846,26 +10706,26 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>29 Mawkynrew</t>
+          <t>22 Nongkrem</t>
         </is>
       </c>
       <c r="E58" t="n">
-        <v>40257</v>
+        <v>40276</v>
       </c>
       <c r="F58" t="n">
-        <v>38802</v>
+        <v>37246</v>
       </c>
       <c r="G58" t="n">
-        <v>1455</v>
+        <v>3030</v>
       </c>
       <c r="N58" t="n">
-        <v>907</v>
+        <v>1341</v>
       </c>
       <c r="O58" t="n">
-        <v>436</v>
+        <v>1622</v>
       </c>
       <c r="P58" t="n">
-        <v>112</v>
+        <v>67</v>
       </c>
       <c r="Q58" t="inlineStr">
         <is>
@@ -10896,26 +10756,26 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>30 Mairang</t>
+          <t>23 Sohiong</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>46252</v>
+        <v>37496</v>
       </c>
       <c r="F59" t="n">
-        <v>44814</v>
+        <v>35223</v>
       </c>
       <c r="G59" t="n">
-        <v>1438</v>
+        <v>2273</v>
       </c>
       <c r="N59" t="n">
-        <v>828</v>
+        <v>1212</v>
       </c>
       <c r="O59" t="n">
-        <v>520</v>
+        <v>968</v>
       </c>
       <c r="P59" t="n">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="Q59" t="inlineStr">
         <is>
@@ -10946,26 +10806,26 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>31 Mawthadraishan</t>
+          <t>24 Mawphlang</t>
         </is>
       </c>
       <c r="E60" t="n">
-        <v>47498</v>
+        <v>38518</v>
       </c>
       <c r="F60" t="n">
-        <v>46333</v>
+        <v>36168</v>
       </c>
       <c r="G60" t="n">
-        <v>1165</v>
+        <v>2350</v>
       </c>
       <c r="N60" t="n">
-        <v>635</v>
+        <v>1507</v>
       </c>
       <c r="O60" t="n">
-        <v>468</v>
+        <v>675</v>
       </c>
       <c r="P60" t="n">
-        <v>62</v>
+        <v>168</v>
       </c>
       <c r="Q60" t="inlineStr">
         <is>
@@ -10996,26 +10856,26 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>32 Nongstoin</t>
+          <t>25 Mawsynram</t>
         </is>
       </c>
       <c r="E61" t="n">
-        <v>48244</v>
+        <v>39984</v>
       </c>
       <c r="F61" t="n">
-        <v>46649</v>
+        <v>37626</v>
       </c>
       <c r="G61" t="n">
-        <v>1595</v>
+        <v>2358</v>
       </c>
       <c r="N61" t="n">
-        <v>1075</v>
+        <v>1483</v>
       </c>
       <c r="O61" t="n">
-        <v>432</v>
+        <v>739</v>
       </c>
       <c r="P61" t="n">
-        <v>88</v>
+        <v>136</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
@@ -11046,26 +10906,26 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>33 Rambrai Jyrngam</t>
+          <t>26 Shella</t>
         </is>
       </c>
       <c r="E62" t="n">
-        <v>43962</v>
+        <v>37925</v>
       </c>
       <c r="F62" t="n">
-        <v>40903</v>
+        <v>35207</v>
       </c>
       <c r="G62" t="n">
-        <v>3059</v>
+        <v>2718</v>
       </c>
       <c r="N62" t="n">
-        <v>1519</v>
+        <v>1558</v>
       </c>
       <c r="O62" t="n">
-        <v>1310</v>
+        <v>1072</v>
       </c>
       <c r="P62" t="n">
-        <v>230</v>
+        <v>88</v>
       </c>
       <c r="Q62" t="inlineStr">
         <is>
@@ -11096,26 +10956,26 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>34 Mawshynrut</t>
+          <t>27 Pynursla</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>45521</v>
+        <v>41748</v>
       </c>
       <c r="F63" t="n">
-        <v>42268</v>
+        <v>39314</v>
       </c>
       <c r="G63" t="n">
-        <v>3253</v>
+        <v>2434</v>
       </c>
       <c r="N63" t="n">
-        <v>1861</v>
+        <v>1941</v>
       </c>
       <c r="O63" t="n">
-        <v>1271</v>
+        <v>390</v>
       </c>
       <c r="P63" t="n">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
@@ -11146,26 +11006,26 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>35 Ranikor</t>
+          <t>28 Sohra</t>
         </is>
       </c>
       <c r="E64" t="n">
-        <v>39247</v>
+        <v>32220</v>
       </c>
       <c r="F64" t="n">
-        <v>37254</v>
+        <v>30532</v>
       </c>
       <c r="G64" t="n">
-        <v>1993</v>
+        <v>1688</v>
       </c>
       <c r="N64" t="n">
-        <v>1216</v>
+        <v>1329</v>
       </c>
       <c r="O64" t="n">
-        <v>705</v>
+        <v>313</v>
       </c>
       <c r="P64" t="n">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="Q64" t="inlineStr">
         <is>
@@ -11196,26 +11056,26 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>36 Mawkyrwat</t>
+          <t>29 Mawkynrew</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>41345</v>
+        <v>40257</v>
       </c>
       <c r="F65" t="n">
-        <v>39870</v>
+        <v>38802</v>
       </c>
       <c r="G65" t="n">
-        <v>1475</v>
+        <v>1455</v>
       </c>
       <c r="N65" t="n">
-        <v>1089</v>
+        <v>907</v>
       </c>
       <c r="O65" t="n">
-        <v>312</v>
+        <v>436</v>
       </c>
       <c r="P65" t="n">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
@@ -11246,26 +11106,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>37 Kharkutta</t>
+          <t>30 Mairang</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>44866</v>
+        <v>46252</v>
       </c>
       <c r="F66" t="n">
-        <v>40784</v>
+        <v>44814</v>
       </c>
       <c r="G66" t="n">
-        <v>4082</v>
+        <v>1438</v>
       </c>
       <c r="N66" t="n">
-        <v>1050</v>
+        <v>828</v>
       </c>
       <c r="O66" t="n">
-        <v>2910</v>
+        <v>520</v>
       </c>
       <c r="P66" t="n">
-        <v>122</v>
+        <v>90</v>
       </c>
       <c r="Q66" t="inlineStr">
         <is>
@@ -11296,26 +11156,26 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>38 Mendipathar</t>
+          <t>31 Mawthadraishan</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>31082</v>
+        <v>47498</v>
       </c>
       <c r="F67" t="n">
-        <v>28184</v>
+        <v>46333</v>
       </c>
       <c r="G67" t="n">
-        <v>2898</v>
+        <v>1165</v>
       </c>
       <c r="N67" t="n">
-        <v>1282</v>
+        <v>635</v>
       </c>
       <c r="O67" t="n">
-        <v>1524</v>
+        <v>468</v>
       </c>
       <c r="P67" t="n">
-        <v>92</v>
+        <v>62</v>
       </c>
       <c r="Q67" t="inlineStr">
         <is>
@@ -11346,26 +11206,26 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>39 Resubelpara</t>
+          <t>32 Nongstoin</t>
         </is>
       </c>
       <c r="E68" t="n">
-        <v>32138</v>
+        <v>48244</v>
       </c>
       <c r="F68" t="n">
-        <v>29834</v>
+        <v>46649</v>
       </c>
       <c r="G68" t="n">
-        <v>2304</v>
+        <v>1595</v>
       </c>
       <c r="N68" t="n">
-        <v>919</v>
+        <v>1075</v>
       </c>
       <c r="O68" t="n">
-        <v>1315</v>
+        <v>432</v>
       </c>
       <c r="P68" t="n">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="Q68" t="inlineStr">
         <is>
@@ -11396,26 +11256,26 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>40 Bajengdoba</t>
+          <t>33 Rambrai Jyrngam</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>35662</v>
+        <v>43962</v>
       </c>
       <c r="F69" t="n">
-        <v>33211</v>
+        <v>40903</v>
       </c>
       <c r="G69" t="n">
-        <v>2451</v>
+        <v>3059</v>
       </c>
       <c r="N69" t="n">
-        <v>1327</v>
+        <v>1519</v>
       </c>
       <c r="O69" t="n">
-        <v>1020</v>
+        <v>1310</v>
       </c>
       <c r="P69" t="n">
-        <v>104</v>
+        <v>230</v>
       </c>
       <c r="Q69" t="inlineStr">
         <is>
@@ -11446,26 +11306,26 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>41 Songsak</t>
+          <t>34 Mawshynrut</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>35518</v>
+        <v>45521</v>
       </c>
       <c r="F70" t="n">
-        <v>33304</v>
+        <v>42268</v>
       </c>
       <c r="G70" t="n">
-        <v>2214</v>
+        <v>3253</v>
       </c>
       <c r="N70" t="n">
-        <v>1069</v>
+        <v>1861</v>
       </c>
       <c r="O70" t="n">
-        <v>1029</v>
+        <v>1271</v>
       </c>
       <c r="P70" t="n">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -11496,26 +11356,26 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>42 Rongjeng</t>
+          <t>35 Ranikor</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>39099</v>
+        <v>39247</v>
       </c>
       <c r="F71" t="n">
-        <v>36444</v>
+        <v>37254</v>
       </c>
       <c r="G71" t="n">
-        <v>2655</v>
+        <v>1993</v>
       </c>
       <c r="N71" t="n">
-        <v>1055</v>
+        <v>1216</v>
       </c>
       <c r="O71" t="n">
-        <v>1361</v>
+        <v>705</v>
       </c>
       <c r="P71" t="n">
-        <v>239</v>
+        <v>72</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
@@ -11546,26 +11406,26 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>43 William Nagar</t>
+          <t>36 Mawkyrwat</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>40150</v>
+        <v>41345</v>
       </c>
       <c r="F72" t="n">
-        <v>35764</v>
+        <v>39870</v>
       </c>
       <c r="G72" t="n">
-        <v>4386</v>
+        <v>1475</v>
       </c>
       <c r="N72" t="n">
-        <v>781</v>
+        <v>1089</v>
       </c>
       <c r="O72" t="n">
-        <v>3371</v>
+        <v>312</v>
       </c>
       <c r="P72" t="n">
-        <v>234</v>
+        <v>74</v>
       </c>
       <c r="Q72" t="inlineStr">
         <is>
@@ -11596,26 +11456,26 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>44 Raksamgre</t>
+          <t>37 Kharkutta</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>33456</v>
+        <v>44866</v>
       </c>
       <c r="F73" t="n">
-        <v>30713</v>
+        <v>40784</v>
       </c>
       <c r="G73" t="n">
-        <v>2743</v>
+        <v>4082</v>
       </c>
       <c r="N73" t="n">
-        <v>1768</v>
+        <v>1050</v>
       </c>
       <c r="O73" t="n">
-        <v>878</v>
+        <v>2910</v>
       </c>
       <c r="P73" t="n">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="Q73" t="inlineStr">
         <is>
@@ -11646,26 +11506,26 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>45 Tikrikilla</t>
+          <t>38 Mendipathar</t>
         </is>
       </c>
       <c r="E74" t="n">
-        <v>38102</v>
+        <v>31082</v>
       </c>
       <c r="F74" t="n">
-        <v>35614</v>
+        <v>28184</v>
       </c>
       <c r="G74" t="n">
-        <v>2488</v>
+        <v>2898</v>
       </c>
       <c r="N74" t="n">
-        <v>1611</v>
+        <v>1282</v>
       </c>
       <c r="O74" t="n">
-        <v>813</v>
+        <v>1524</v>
       </c>
       <c r="P74" t="n">
-        <v>64</v>
+        <v>92</v>
       </c>
       <c r="Q74" t="inlineStr">
         <is>
@@ -11696,26 +11556,26 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>46 Phulbari</t>
+          <t>39 Resubelpara</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>35902</v>
+        <v>32138</v>
       </c>
       <c r="F75" t="n">
-        <v>33941</v>
+        <v>29834</v>
       </c>
       <c r="G75" t="n">
-        <v>1961</v>
+        <v>2304</v>
       </c>
       <c r="N75" t="n">
-        <v>1256</v>
+        <v>919</v>
       </c>
       <c r="O75" t="n">
-        <v>653</v>
+        <v>1315</v>
       </c>
       <c r="P75" t="n">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="Q75" t="inlineStr">
         <is>
@@ -11746,26 +11606,26 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>47 Rajabala</t>
+          <t>40 Bajengdoba</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>38778</v>
+        <v>35662</v>
       </c>
       <c r="F76" t="n">
-        <v>37092</v>
+        <v>33211</v>
       </c>
       <c r="G76" t="n">
-        <v>1686</v>
+        <v>2451</v>
       </c>
       <c r="N76" t="n">
-        <v>926</v>
+        <v>1327</v>
       </c>
       <c r="O76" t="n">
-        <v>659</v>
+        <v>1020</v>
       </c>
       <c r="P76" t="n">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="Q76" t="inlineStr">
         <is>
@@ -11796,26 +11656,26 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>48 Selsella</t>
+          <t>41 Songsak</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>39293</v>
+        <v>35518</v>
       </c>
       <c r="F77" t="n">
-        <v>37294</v>
+        <v>33304</v>
       </c>
       <c r="G77" t="n">
-        <v>1999</v>
+        <v>2214</v>
       </c>
       <c r="N77" t="n">
-        <v>1200</v>
+        <v>1069</v>
       </c>
       <c r="O77" t="n">
-        <v>726</v>
+        <v>1029</v>
       </c>
       <c r="P77" t="n">
-        <v>73</v>
+        <v>116</v>
       </c>
       <c r="Q77" t="inlineStr">
         <is>
@@ -11846,26 +11706,26 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>49 Dadenggre</t>
+          <t>42 Rongjeng</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>39880</v>
+        <v>39099</v>
       </c>
       <c r="F78" t="n">
-        <v>37073</v>
+        <v>36444</v>
       </c>
       <c r="G78" t="n">
-        <v>2807</v>
+        <v>2655</v>
       </c>
       <c r="N78" t="n">
-        <v>1870</v>
+        <v>1055</v>
       </c>
       <c r="O78" t="n">
-        <v>851</v>
+        <v>1361</v>
       </c>
       <c r="P78" t="n">
-        <v>86</v>
+        <v>239</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
@@ -11896,26 +11756,26 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>50 North Tura</t>
+          <t>43 William Nagar</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>36631</v>
+        <v>40150</v>
       </c>
       <c r="F79" t="n">
-        <v>32415</v>
+        <v>35764</v>
       </c>
       <c r="G79" t="n">
-        <v>4216</v>
+        <v>4386</v>
       </c>
       <c r="N79" t="n">
-        <v>1526</v>
+        <v>781</v>
       </c>
       <c r="O79" t="n">
-        <v>2579</v>
+        <v>3371</v>
       </c>
       <c r="P79" t="n">
-        <v>111</v>
+        <v>234</v>
       </c>
       <c r="Q79" t="inlineStr">
         <is>
@@ -11946,26 +11806,26 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>51 South Tura</t>
+          <t>44 Raksamgre</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>35796</v>
+        <v>33456</v>
       </c>
       <c r="F80" t="n">
-        <v>30784</v>
+        <v>30713</v>
       </c>
       <c r="G80" t="n">
-        <v>5012</v>
+        <v>2743</v>
       </c>
       <c r="N80" t="n">
-        <v>1938</v>
+        <v>1768</v>
       </c>
       <c r="O80" t="n">
-        <v>3009</v>
+        <v>878</v>
       </c>
       <c r="P80" t="n">
-        <v>65</v>
+        <v>97</v>
       </c>
       <c r="Q80" t="inlineStr">
         <is>
@@ -11996,26 +11856,26 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>52 Rangsakona</t>
+          <t>45 Tikrikilla</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>40914</v>
+        <v>38102</v>
       </c>
       <c r="F81" t="n">
-        <v>37742</v>
+        <v>35614</v>
       </c>
       <c r="G81" t="n">
-        <v>3172</v>
+        <v>2488</v>
       </c>
       <c r="N81" t="n">
-        <v>1747</v>
+        <v>1611</v>
       </c>
       <c r="O81" t="n">
-        <v>1327</v>
+        <v>813</v>
       </c>
       <c r="P81" t="n">
-        <v>98</v>
+        <v>64</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
@@ -12046,26 +11906,26 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>53 Ampati</t>
+          <t>46 Phulbari</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>35573</v>
+        <v>35902</v>
       </c>
       <c r="F82" t="n">
-        <v>34326</v>
+        <v>33941</v>
       </c>
       <c r="G82" t="n">
-        <v>1247</v>
+        <v>1961</v>
       </c>
       <c r="N82" t="n">
-        <v>755</v>
+        <v>1256</v>
       </c>
       <c r="O82" t="n">
-        <v>406</v>
+        <v>653</v>
       </c>
       <c r="P82" t="n">
-        <v>86</v>
+        <v>52</v>
       </c>
       <c r="Q82" t="inlineStr">
         <is>
@@ -12096,26 +11956,26 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>54 Mahendraganj</t>
+          <t>47 Rajabala</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>39339</v>
+        <v>38778</v>
       </c>
       <c r="F83" t="n">
-        <v>37887</v>
+        <v>37092</v>
       </c>
       <c r="G83" t="n">
-        <v>1452</v>
+        <v>1686</v>
       </c>
       <c r="N83" t="n">
-        <v>812</v>
+        <v>926</v>
       </c>
       <c r="O83" t="n">
-        <v>582</v>
+        <v>659</v>
       </c>
       <c r="P83" t="n">
-        <v>58</v>
+        <v>101</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -12146,26 +12006,26 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>55 Salmanpara</t>
+          <t>48 Selsella</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>33971</v>
+        <v>39293</v>
       </c>
       <c r="F84" t="n">
-        <v>32458</v>
+        <v>37294</v>
       </c>
       <c r="G84" t="n">
-        <v>1513</v>
+        <v>1999</v>
       </c>
       <c r="N84" t="n">
-        <v>911</v>
+        <v>1200</v>
       </c>
       <c r="O84" t="n">
-        <v>440</v>
+        <v>726</v>
       </c>
       <c r="P84" t="n">
-        <v>162</v>
+        <v>73</v>
       </c>
       <c r="Q84" t="inlineStr">
         <is>
@@ -12196,26 +12056,26 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>56 Gambegre</t>
+          <t>49 Dadenggre</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>34857</v>
+        <v>39880</v>
       </c>
       <c r="F85" t="n">
-        <v>33072</v>
+        <v>37073</v>
       </c>
       <c r="G85" t="n">
-        <v>1785</v>
+        <v>2807</v>
       </c>
       <c r="N85" t="n">
-        <v>899</v>
+        <v>1870</v>
       </c>
       <c r="O85" t="n">
-        <v>716</v>
+        <v>851</v>
       </c>
       <c r="P85" t="n">
-        <v>170</v>
+        <v>86</v>
       </c>
       <c r="Q85" t="inlineStr">
         <is>
@@ -12246,26 +12106,26 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>57 Dalu</t>
+          <t>50 North Tura</t>
         </is>
       </c>
       <c r="E86" t="n">
-        <v>23305</v>
+        <v>36631</v>
       </c>
       <c r="F86" t="n">
-        <v>21642</v>
+        <v>32415</v>
       </c>
       <c r="G86" t="n">
-        <v>1663</v>
+        <v>4216</v>
       </c>
       <c r="N86" t="n">
-        <v>872</v>
+        <v>1526</v>
       </c>
       <c r="O86" t="n">
-        <v>663</v>
+        <v>2579</v>
       </c>
       <c r="P86" t="n">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="Q86" t="inlineStr">
         <is>
@@ -12296,26 +12156,26 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>58 Rongara Siju</t>
+          <t>51 South Tura</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>38179</v>
+        <v>35796</v>
       </c>
       <c r="F87" t="n">
-        <v>34882</v>
+        <v>30784</v>
       </c>
       <c r="G87" t="n">
-        <v>3297</v>
+        <v>5012</v>
       </c>
       <c r="N87" t="n">
-        <v>1261</v>
+        <v>1938</v>
       </c>
       <c r="O87" t="n">
-        <v>1798</v>
+        <v>3009</v>
       </c>
       <c r="P87" t="n">
-        <v>238</v>
+        <v>65</v>
       </c>
       <c r="Q87" t="inlineStr">
         <is>
@@ -12346,26 +12206,26 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>59 Chokpot</t>
+          <t>52 Rangsakona</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>35921</v>
+        <v>40914</v>
       </c>
       <c r="F88" t="n">
-        <v>33400</v>
+        <v>37742</v>
       </c>
       <c r="G88" t="n">
-        <v>2521</v>
+        <v>3172</v>
       </c>
       <c r="N88" t="n">
-        <v>1270</v>
+        <v>1747</v>
       </c>
       <c r="O88" t="n">
-        <v>1151</v>
+        <v>1327</v>
       </c>
       <c r="P88" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="Q88" t="inlineStr">
         <is>
@@ -12396,38 +12256,388 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
+          <t>53 Ampati</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>35573</v>
+      </c>
+      <c r="F89" t="n">
+        <v>34326</v>
+      </c>
+      <c r="G89" t="n">
+        <v>1247</v>
+      </c>
+      <c r="N89" t="n">
+        <v>755</v>
+      </c>
+      <c r="O89" t="n">
+        <v>406</v>
+      </c>
+      <c r="P89" t="n">
+        <v>86</v>
+      </c>
+      <c r="Q89" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>54 Mahendraganj</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>39339</v>
+      </c>
+      <c r="F90" t="n">
+        <v>37887</v>
+      </c>
+      <c r="G90" t="n">
+        <v>1452</v>
+      </c>
+      <c r="N90" t="n">
+        <v>812</v>
+      </c>
+      <c r="O90" t="n">
+        <v>582</v>
+      </c>
+      <c r="P90" t="n">
+        <v>58</v>
+      </c>
+      <c r="Q90" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>55 Salmanpara</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>33971</v>
+      </c>
+      <c r="F91" t="n">
+        <v>32458</v>
+      </c>
+      <c r="G91" t="n">
+        <v>1513</v>
+      </c>
+      <c r="N91" t="n">
+        <v>911</v>
+      </c>
+      <c r="O91" t="n">
+        <v>440</v>
+      </c>
+      <c r="P91" t="n">
+        <v>162</v>
+      </c>
+      <c r="Q91" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>56 Gambegre</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>34857</v>
+      </c>
+      <c r="F92" t="n">
+        <v>33072</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1785</v>
+      </c>
+      <c r="N92" t="n">
+        <v>899</v>
+      </c>
+      <c r="O92" t="n">
+        <v>716</v>
+      </c>
+      <c r="P92" t="n">
+        <v>170</v>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>57 Dalu</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>23305</v>
+      </c>
+      <c r="F93" t="n">
+        <v>21642</v>
+      </c>
+      <c r="G93" t="n">
+        <v>1663</v>
+      </c>
+      <c r="N93" t="n">
+        <v>872</v>
+      </c>
+      <c r="O93" t="n">
+        <v>663</v>
+      </c>
+      <c r="P93" t="n">
+        <v>128</v>
+      </c>
+      <c r="Q93" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>58 Rongara Siju</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>38179</v>
+      </c>
+      <c r="F94" t="n">
+        <v>34882</v>
+      </c>
+      <c r="G94" t="n">
+        <v>3297</v>
+      </c>
+      <c r="N94" t="n">
+        <v>1261</v>
+      </c>
+      <c r="O94" t="n">
+        <v>1798</v>
+      </c>
+      <c r="P94" t="n">
+        <v>238</v>
+      </c>
+      <c r="Q94" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>59 Chokpot</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>35921</v>
+      </c>
+      <c r="F95" t="n">
+        <v>33400</v>
+      </c>
+      <c r="G95" t="n">
+        <v>2521</v>
+      </c>
+      <c r="N95" t="n">
+        <v>1270</v>
+      </c>
+      <c r="O95" t="n">
+        <v>1151</v>
+      </c>
+      <c r="P95" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q95" t="inlineStr">
+        <is>
+          <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
+        </is>
+      </c>
+      <c r="R95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>constituencies</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>ac</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
           <t>60 Baghmara</t>
         </is>
       </c>
-      <c r="E89" t="n">
+      <c r="E96" t="n">
         <v>36388</v>
       </c>
-      <c r="F89" t="n">
+      <c r="F96" t="n">
         <v>34367</v>
       </c>
-      <c r="G89" t="n">
+      <c r="G96" t="n">
         <v>2021</v>
       </c>
-      <c r="N89" t="n">
+      <c r="N96" t="n">
         <v>1052</v>
       </c>
-      <c r="O89" t="n">
+      <c r="O96" t="n">
         <v>833</v>
       </c>
-      <c r="P89" t="n">
+      <c r="P96" t="n">
         <v>136</v>
       </c>
-      <c r="Q89" t="inlineStr">
+      <c r="Q96" t="inlineStr">
         <is>
           <t>Election Department, Government of Meghalaya (Chief Electoral Officer), press note No. EL.63/2026/29 of 5 August 2026 with the SIR status report by constituency</t>
         </is>
       </c>
-      <c r="R89" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S89" t="inlineStr">
+      <c r="R96" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S96" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>